<commit_message>
Quitar foto de cortinas de seguridad duplicada en 9 estaciones
Se elimina la foto de cortinas de seguridad de las 7 estaciones
Moose/Scorpion restantes (se conserva solo en Final Assy Moose) y de
Gasket Attach Gecko y Cartridge Attach Gecko, dejando esas dos
posiciones de foto en blanco. Se regeneraron los PDF individuales
afectados y el PDF combinado de las 16 estaciones.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtjxNEToLwFA6ZBpe5Zyeg
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Back_Assy_Moose_Scorpion.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Back_Assy_Moose_Scorpion.xlsx
@@ -1784,7 +1784,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="34082" t="29556" r="36328" b="57813"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1828,7 +1828,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1877,7 +1877,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1921,7 +1921,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1967,7 +1967,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="34082" t="29556" r="36328" b="57813"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -2048,34 +2048,6 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
-      <colOff>95250</colOff>
-      <row>80</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="4953000" cy="3590925"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
       <col>11</col>
       <colOff>95250</colOff>
       <row>80</row>
@@ -2088,35 +2060,7 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>95250</colOff>
-      <row>90</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="4953000" cy="3590925"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2144,7 +2088,7 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2172,7 +2116,7 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2200,7 +2144,7 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>

</xml_diff>